<commit_message>
Agregar boton "Ver detalle" y corregir las tildes de los titulos del informe
Panel
- Cada tarjeta del Kanban suma un boton explicito "Ver detalle" junto a
  Editar y Eliminar. El nombre del candidato sigue siendo un enlace, pero
  como unico acceso no era descubrible.

Titulos del informe
- El generador de plantillas producia las columnas "Areas de mejora" y
  "Conclusion" sin tilde, y de ahi salen las secciones del informe. Se
  corrigen en el generador y se regeneran las plantillas de las cuatro
  familias. Tambien se corrigen los nombres "Atencion al Cliente" y
  "Administracion" usados como titulo de la pauta, que habian quedado
  desalineados con los nombres ya migrados en la base.
- Nuevo migrarTitulosInformes.js: los titulos se guardan junto al informe,
  asi que corregir las plantillas no arreglaba los informes existentes.
  El script los actualiza conservando el contenido de cada seccion, y es
  idempotente.
</commit_message>
<xml_diff>
--- a/backend/plantillas/administracion/plantilla_informe.xlsx
+++ b/backend/plantillas/administracion/plantilla_informe.xlsx
@@ -22,16 +22,16 @@
     <t>Fortalezas</t>
   </si>
   <si>
-    <t>Areas de mejora</t>
-  </si>
-  <si>
-    <t>Conclusion</t>
+    <t>Áreas de mejora</t>
+  </si>
+  <si>
+    <t>Conclusión</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>Administracion</t>
+    <t>Administración</t>
   </si>
 </sst>
 </file>

</xml_diff>